<commit_message>
feat: big update on archives
</commit_message>
<xml_diff>
--- a/04 - Pointing/01 - LP's/ApontamentoRodrigo.xlsx
+++ b/04 - Pointing/01 - LP's/ApontamentoRodrigo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,194 +443,402 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LP053953</t>
+          <t>LP053407</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LP053951</t>
+          <t>LP053410</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LP053950</t>
+          <t>LP053412</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LP053949</t>
+          <t>LP053411</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LP053948</t>
+          <t>LP053414</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LP053940</t>
+          <t>LP053415</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LP053804</t>
+          <t>LP053418</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LP053799</t>
+          <t>LP053419</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LP053828</t>
+          <t>LP052787</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LP053893</t>
+          <t>LP053085</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LP053827</t>
+          <t>LP053086</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LP053883</t>
+          <t>LP053084</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Line created!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LP054158</t>
+          <t>LP053083</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LP doesn't exist!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LP054161</t>
+          <t>LP053082</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LP doesn't exist!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LP054160</t>
+          <t>LP053081</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LP doesn't exist!</t>
+          <t>Apointing created!</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LP054159</t>
+          <t>LP053080</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LP doesn't exist!</t>
-        </is>
-      </c>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LP052899</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LP053055</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LP053053</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LP053054</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LP053037</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LP053036</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LP053035</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LP053034</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LP053033</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LP053032</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LP053029</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LP052977</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Apointing created!</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LP052978</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LP053426</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LP053427</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LP053428</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LP052990</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>LP052989</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LP052991</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LP052992</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>